<commit_message>
feat: implementar y probar las reglas de aprobación, y documentar el alcance real
- automation_engine.py pasa de imprimir una simulación a implementar las reglas
  R1-R5 del blueprint: valida contra el maestro de facturas, aplica los topes
  de aprobación y escribe una bitácora auditable de cada dictamen.
- Se unifica el tope de autoaprobación en S/ 50 (el motor usaba S/ 30 mientras
  la app y la documentación decían S/ 50).
- Nueva suite de 9 pruebas sobre los límites de cada regla.
- Los datos de prueba usaban nombres de empresas reales como clientes
  ficticios; se reemplazaron por entidades claramente inventadas.
- README reescrito: distingue qué es código ejecutable y qué es especificación
  de Power Platform, declara que no hay despliegue en un tenant y cambia la
  tabla de "eficiencia" por criterios de diseño.
- Añadido LICENSE (MIT), que el README ya declaraba, y actualizado el ciclo.
</commit_message>
<xml_diff>
--- a/data/FacturasEmitidas.xlsx
+++ b/data/FacturasEmitidas.xlsx
@@ -139,31 +139,31 @@
     <t>CLI-810</t>
   </si>
   <si>
-    <t>Minera Las Bambas S.A.</t>
+    <t>Minera Altoandina S.A.C.</t>
   </si>
   <si>
     <t>Juan Carlos Pérez Gómez</t>
   </si>
   <si>
-    <t>Distribuidora Lima Norte S.A.C.</t>
+    <t>Distribuidora Vista Norte S.A.C.</t>
   </si>
   <si>
     <t>María Elena Rodríguez Prado</t>
   </si>
   <si>
-    <t>Constructora Graña &amp; Asociados</t>
+    <t>Constructora Ribera del Norte S.A.C.</t>
   </si>
   <si>
     <t>Carlos Alberto Mendoza Solís</t>
   </si>
   <si>
-    <t>Textil San Pedro E.I.R.L.</t>
+    <t>Textil Santa Aurora E.I.R.L.</t>
   </si>
   <si>
     <t>Lucía Valeria Quispe Huamán</t>
   </si>
   <si>
-    <t>Corporación Minera del Sur S.A.C.</t>
+    <t>Corporación Minera Pampa Azul S.A.C.</t>
   </si>
   <si>
     <t>Roberto Alonso Chávez Ramos</t>

</xml_diff>